<commit_message>
Add western mound sites and western natural mound look-alike fields
docs/west-mound-training-sites.csv: 7 western sites (Hohokam platform
mounds in Arizona, Plains village midden mounds in North Dakota).
docs/west-natural-mound-lookalikes.csv: 8 natural mound fields (Mima,
hogwallow, pimple and biscuit-scabland mounds) to tour and answer Not real.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V6AhsWjuRrwGnXBnM99QwT
</commit_message>
<xml_diff>
--- a/docs/all-training-sites.xlsx
+++ b/docs/all-training-sites.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G354"/>
+  <dimension ref="A1:G369"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11178,6 +11178,445 @@
         </is>
       </c>
     </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>Pueblo Grande platform mound, Phoenix (AZ)</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Mounds</t>
+        </is>
+      </c>
+      <c r="C355" t="n">
+        <v>33.4456</v>
+      </c>
+      <c r="D355" t="n">
+        <v>-111.98403</v>
+      </c>
+      <c r="E355" t="inlineStr"/>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>5: 7 western mound sites</t>
+        </is>
+      </c>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>USGS place-names (GNIS) position</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>Mesa Grande platform mound, Mesa (AZ)</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Mounds</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr"/>
+      <c r="D356" t="inlineStr"/>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>Mesa Grande Cultural Park, Mesa, Arizona</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>5: 7 western mound sites</t>
+        </is>
+      </c>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>found by name lookup when toured</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>Casa Grande Ruins (AZ)</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Mounds</t>
+        </is>
+      </c>
+      <c r="C357" t="n">
+        <v>32.99703</v>
+      </c>
+      <c r="D357" t="n">
+        <v>-111.53254</v>
+      </c>
+      <c r="E357" t="inlineStr"/>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>5: 7 western mound sites</t>
+        </is>
+      </c>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t>USGS place-names (GNIS) position</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>Gatlin Site platform mounds, Gila Bend (AZ)</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Mounds</t>
+        </is>
+      </c>
+      <c r="C358" t="n">
+        <v>32.98639</v>
+      </c>
+      <c r="D358" t="n">
+        <v>-112.70194</v>
+      </c>
+      <c r="E358" t="inlineStr"/>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>5: 7 western mound sites</t>
+        </is>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>USGS place-names (GNIS) position</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>Snaketown, Hohokam Pima NM (AZ)</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Mounds</t>
+        </is>
+      </c>
+      <c r="C359" t="n">
+        <v>33.18714</v>
+      </c>
+      <c r="D359" t="n">
+        <v>-111.91927</v>
+      </c>
+      <c r="E359" t="inlineStr"/>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>5: 7 western mound sites</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>USGS place-names (GNIS) position</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>Double Ditch village midden mounds (ND)</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Mounds</t>
+        </is>
+      </c>
+      <c r="C360" t="n">
+        <v>46.93521</v>
+      </c>
+      <c r="D360" t="n">
+        <v>-100.89683</v>
+      </c>
+      <c r="E360" t="inlineStr"/>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>5: 7 western mound sites</t>
+        </is>
+      </c>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>historical marker position (site in view; use the 1000 m size)</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>Knife River Indian Villages (ND)</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Mounds</t>
+        </is>
+      </c>
+      <c r="C361" t="n">
+        <v>47.3539</v>
+      </c>
+      <c r="D361" t="n">
+        <v>-101.38572</v>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>Big Hidatsa Village Site, Knife River Indian Villages, North Dakota</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>5: 7 western mound sites</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>USGS place-names (GNIS) position</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>NATURAL: Mima Mounds Natural Area Preserve (WA) - answer Not real</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Mounds</t>
+        </is>
+      </c>
+      <c r="C362" t="n">
+        <v>46.89704</v>
+      </c>
+      <c r="D362" t="n">
+        <v>-123.0507</v>
+      </c>
+      <c r="E362" t="inlineStr"/>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>6: 8 western natural mound fields (answer Not real)</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>USGS place-names (GNIS) position</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>NATURAL: Glacial Heritage Preserve mima mounds (WA) - answer Not real</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Mounds</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr"/>
+      <c r="D363" t="inlineStr"/>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>Glacial Heritage Preserve, Thurston County, Washington</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>6: 8 western natural mound fields (answer Not real)</t>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>found by name lookup when toured</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>NATURAL: Turnbull NWR biscuit scabland mounds (WA) - answer Not real</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Mounds</t>
+        </is>
+      </c>
+      <c r="C364" t="n">
+        <v>47.42252</v>
+      </c>
+      <c r="D364" t="n">
+        <v>-117.57129</v>
+      </c>
+      <c r="E364" t="inlineStr"/>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>6: 8 western natural mound fields (answer Not real)</t>
+        </is>
+      </c>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>USGS place-names (GNIS) position</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>NATURAL: Upper Table Rock mounds (OR) - answer Not real</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Mounds</t>
+        </is>
+      </c>
+      <c r="C365" t="n">
+        <v>42.47574</v>
+      </c>
+      <c r="D365" t="n">
+        <v>-122.9194</v>
+      </c>
+      <c r="E365" t="inlineStr"/>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>6: 8 western natural mound fields (answer Not real)</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>USGS place-names (GNIS) position</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>NATURAL: Jepson Prairie hogwallow mounds (CA) - answer Not real</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Mounds</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr"/>
+      <c r="D366" t="inlineStr"/>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>Jepson Prairie Preserve, Solano County, California</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>6: 8 western natural mound fields (answer Not real)</t>
+        </is>
+      </c>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>found by name lookup when toured</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>NATURAL: Merced Vernal Pools mounds (CA) - answer Not real</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Mounds</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr"/>
+      <c r="D367" t="inlineStr"/>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>Merced Vernal Pools and Grassland Reserve, California</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>6: 8 western natural mound fields (answer Not real)</t>
+        </is>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>found by name lookup when toured</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>NATURAL: Santa Rosa Plateau mima mounds (CA) - answer Not real</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Mounds</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr"/>
+      <c r="D368" t="inlineStr"/>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>Santa Rosa Plateau Ecological Reserve, California</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>6: 8 western natural mound fields (answer Not real)</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>found by name lookup when toured</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>NATURAL: Attwater Prairie Chicken NWR pimple mounds (TX) - answer Not real</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Mounds</t>
+        </is>
+      </c>
+      <c r="C369" t="n">
+        <v>29.69058</v>
+      </c>
+      <c r="D369" t="n">
+        <v>-96.27819</v>
+      </c>
+      <c r="E369" t="inlineStr"/>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>6: 8 western natural mound fields (answer Not real)</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>USGS place-names (GNIS) position</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>